<commit_message>
feat: liquidacion por dias reactivada para pendientes/bajas, columna Fecha de Liquidacion para cobradas, vista diaria en Ventas por Sector y Bajas, y Proyeccion 12 meses alineada al modelo mes-cerrado/mes-actual
</commit_message>
<xml_diff>
--- a/static/plantillas/PLANTILLA_4_Pilares.xlsx
+++ b/static/plantillas/PLANTILLA_4_Pilares.xlsx
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -103,6 +103,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A136"/>
+  <dimension ref="A1:A147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1146,9 +1148,6 @@
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="inlineStr"/>
-    </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
@@ -1177,9 +1176,6 @@
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" t="inlineStr"/>
-    </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
@@ -1208,9 +1204,6 @@
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" t="inlineStr"/>
-    </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
@@ -1222,6 +1215,71 @@
       <c r="A136" t="inlineStr">
         <is>
           <t>de cada sector).</t>
+        </is>
+      </c>
+    </row>
+    <row r="137"/>
+    <row r="138">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t>20. COLUMNA 'Fecha de Liquidación' (solo ventas COBRADAS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="9" t="inlineStr">
+        <is>
+          <t>Toda venta ya Cobrada debería tener una Fecha de Liquidación: es la fecha en la que</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="9" t="inlineStr">
+        <is>
+          <t>realmente entra el dinero en caja, y es la que BETTY usa para ubicar esa venta (mes y día)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="9" t="inlineStr">
+        <is>
+          <t>en el gráfico 'Ingresos, Gastos y Evolución de Caja' (pestaña Análisis Detallado) — no su</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="9" t="inlineStr">
+        <is>
+          <t>columna Fecha. Si la dejas vacía, se usará la columna Fecha en su lugar, y la app mostrará</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="9" t="inlineStr">
+        <is>
+          <t>un aviso con cuántas ventas cobradas no tienen Fecha de Liquidación, ya que puede distorsionar</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="inlineStr">
+        <is>
+          <t>los resultados (la venta aparecería antes o después de cuando realmente se cobró).</t>
+        </is>
+      </c>
+    </row>
+    <row r="145"/>
+    <row r="146">
+      <c r="A146" s="9" t="inlineStr">
+        <is>
+          <t>Esta columna NO aplica a ventas Pendientes: esas se siguen proyectando según la Fecha de</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="inlineStr">
+        <is>
+          <t>Activación y la Liquidación (días del mes) configurada por comercializadora (ver punto 18).</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1395,6 +1453,11 @@
       </c>
       <c r="Z1" s="7" t="inlineStr">
         <is>
+          <t>Fecha de Liquidación</t>
+        </is>
+      </c>
+      <c r="AA1" s="7" t="inlineStr">
+        <is>
           <t>Sector</t>
         </is>
       </c>
@@ -1523,6 +1586,11 @@
       <c r="R3" t="n">
         <v>24</v>
       </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1605,6 +1673,11 @@
       <c r="R4" t="n">
         <v>18</v>
       </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1701,7 +1774,7 @@
           <t>Pagado</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>Energía</t>
         </is>
@@ -1884,6 +1957,11 @@
       <c r="R9" t="n">
         <v>0</v>
       </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1966,6 +2044,11 @@
       <c r="R10" t="n">
         <v>20</v>
       </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2062,7 +2145,7 @@
           <t>Pagado</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="AA12" t="inlineStr">
         <is>
           <t>Energía</t>
         </is>
@@ -2254,6 +2337,11 @@
           <t>2026-07-10</t>
         </is>
       </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2387,7 +2475,7 @@
           <t>Pagado</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t>Energía</t>
         </is>
@@ -2419,7 +2507,7 @@
     <dataValidation sqref="U2:U300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Luz,Gas"</formula1>
     </dataValidation>
-    <dataValidation sqref="Z2:Z300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AA2:AA300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Energía,Telefonía,Placas Solares,Alarmas"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>